<commit_message>
bugs mentioned in bug report are fixed
</commit_message>
<xml_diff>
--- a/docs/qa_guides/Frontend_Bugs_and_Refactoring_Template(AutoRecovered).xlsx
+++ b/docs/qa_guides/Frontend_Bugs_and_Refactoring_Template(AutoRecovered).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1.STUDY\FYP\Main\Philbox\docs\qa_guides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E774D0-1845-43F1-A473-A7A33DFECB4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC70E29-6C17-4DDA-82FE-7D2D59B0265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="292">
   <si>
     <t>Bug ID</t>
   </si>
@@ -823,6 +823,192 @@
     <t>20nd Feb, 2026</t>
   </si>
   <si>
+    <t>C-006</t>
+  </si>
+  <si>
+    <t>Notification drop down on customer dashboard</t>
+  </si>
+  <si>
+    <t>The minimum screen is 280 and the notification drop down goes out of sight</t>
+  </si>
+  <si>
+    <t>Make it visible and responsive</t>
+  </si>
+  <si>
+    <t>22nd Feb,2026</t>
+  </si>
+  <si>
+    <t>23rd Feb, 2026</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\customer-page-notification-dropdorn.PNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Dashboard cards </t>
+  </si>
+  <si>
+    <t>The minimum screen is 280 and the cards icon goes out of cards.</t>
+  </si>
+  <si>
+    <t>Make it with within the cards</t>
+  </si>
+  <si>
+    <t>Must be adjusted according to the cards size.</t>
+  </si>
+  <si>
+    <t>23rd Feb,2026</t>
+  </si>
+  <si>
+    <t>24th Feb, 2026</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\customer-Dasbboard-cards.PNG</t>
+  </si>
+  <si>
+    <t>C-008</t>
+  </si>
+  <si>
+    <t>C-007</t>
+  </si>
+  <si>
+    <t>Customer Medicine detail page</t>
+  </si>
+  <si>
+    <t>The minimum screen is 280 and the buy now and cadd to cart buttons and other things goes out of the card</t>
+  </si>
+  <si>
+    <t>Make it responsive</t>
+  </si>
+  <si>
+    <t>Must be adjusted according to the card size</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\customer-medicine-details-page.PNG</t>
+  </si>
+  <si>
+    <t>24th Feb,2026</t>
+  </si>
+  <si>
+    <t>25th Feb, 2026</t>
+  </si>
+  <si>
+    <t>C-009</t>
+  </si>
+  <si>
+    <t>Customer order detail page</t>
+  </si>
+  <si>
+    <t>the minimum screen is 280 and the card size miss matched</t>
+  </si>
+  <si>
+    <t>make it responsive</t>
+  </si>
+  <si>
+    <t>Must be adjusted dso that in small screen all cards have same width</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\Customer-order-detail-page.PNG</t>
+  </si>
+  <si>
+    <t>23th Feb,2026</t>
+  </si>
+  <si>
+    <t>C-0010</t>
+  </si>
+  <si>
+    <t>Customer Appointment page botton size</t>
+  </si>
+  <si>
+    <t>The buttons on the appointment cards are of unequal lengths make their width equal when the are in small screen</t>
+  </si>
+  <si>
+    <t>make them of equal width</t>
+  </si>
+  <si>
+    <t>Must be adjusted so that in small screen they seem to be of equal width</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\customer-appointment-page-button size.PNG</t>
+  </si>
+  <si>
+    <t>C-0011</t>
+  </si>
+  <si>
+    <t>Customer book Appointment cards and timeline</t>
+  </si>
+  <si>
+    <t>the min screen size is 280 and the cards of search bar and appointment width mismatched and the time line also goes out of sight</t>
+  </si>
+  <si>
+    <t>must be adjusted to equal widths also time line should be visible</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\Customer-book-appointment responsiveness.PNG</t>
+  </si>
+  <si>
+    <t>C-0012</t>
+  </si>
+  <si>
+    <t>Customer Profile page security tab</t>
+  </si>
+  <si>
+    <t>the min screen size is 280 and the button goes out of the card</t>
+  </si>
+  <si>
+    <t>when the screen size is small the button should be inside the card</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\customer-profile-security-tab.PNG</t>
+  </si>
+  <si>
+    <t>D-001</t>
+  </si>
+  <si>
+    <t>Doctor Registration page logo</t>
+  </si>
+  <si>
+    <t>Ux</t>
+  </si>
+  <si>
+    <t>the logo of vite is shown instead of philbox logo</t>
+  </si>
+  <si>
+    <t>adjust the logo of philbox</t>
+  </si>
+  <si>
+    <t>must show the logo of philbox</t>
+  </si>
+  <si>
+    <t>bugs\screenshots\doctor-registration-page.PNG</t>
+  </si>
+  <si>
+    <t>D-002</t>
+  </si>
+  <si>
+    <t>Doctor login page logo</t>
+  </si>
+  <si>
+    <t>D-003</t>
+  </si>
+  <si>
+    <t>Doctor complete profile</t>
+  </si>
+  <si>
+    <t>ux</t>
+  </si>
+  <si>
+    <t>D-004</t>
+  </si>
+  <si>
+    <t>password and confirm password text bxes size mismatched</t>
+  </si>
+  <si>
+    <t>must be adjusted</t>
+  </si>
+  <si>
+    <t>the size of the textboxes must be responsive and well managed</t>
+  </si>
+  <si>
     <t>Fixed</t>
   </si>
 </sst>
@@ -830,7 +1016,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -858,6 +1044,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1191,12 +1383,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="13" width="25" customWidth="1"/>
+    <col min="3" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="13" width="25" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
@@ -1281,7 +1475,7 @@
         <v>27</v>
       </c>
       <c r="J2" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>28</v>
@@ -1325,7 +1519,7 @@
         <v>27</v>
       </c>
       <c r="J3" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>33</v>
@@ -1369,7 +1563,7 @@
         <v>27</v>
       </c>
       <c r="J4" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>45</v>
@@ -1413,7 +1607,7 @@
         <v>27</v>
       </c>
       <c r="J5" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>52</v>
@@ -1457,7 +1651,7 @@
         <v>27</v>
       </c>
       <c r="J6" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>59</v>
@@ -1501,7 +1695,7 @@
         <v>27</v>
       </c>
       <c r="J7" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>65</v>
@@ -1545,7 +1739,7 @@
         <v>27</v>
       </c>
       <c r="J8" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>70</v>
@@ -1589,7 +1783,7 @@
         <v>78</v>
       </c>
       <c r="J9" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>79</v>
@@ -1633,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="J10" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>87</v>
@@ -1677,7 +1871,7 @@
         <v>92</v>
       </c>
       <c r="J11" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>93</v>
@@ -1721,7 +1915,7 @@
         <v>92</v>
       </c>
       <c r="J12" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>98</v>
@@ -1765,7 +1959,7 @@
         <v>27</v>
       </c>
       <c r="J13" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>103</v>
@@ -1809,7 +2003,7 @@
         <v>27</v>
       </c>
       <c r="J14" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>109</v>
@@ -1853,7 +2047,7 @@
         <v>92</v>
       </c>
       <c r="J15" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>114</v>
@@ -1897,7 +2091,7 @@
         <v>27</v>
       </c>
       <c r="J16" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>119</v>
@@ -1941,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="J17" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>123</v>
@@ -1985,7 +2179,7 @@
         <v>78</v>
       </c>
       <c r="J18" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>129</v>
@@ -2029,7 +2223,7 @@
         <v>27</v>
       </c>
       <c r="J19" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>133</v>
@@ -2073,7 +2267,7 @@
         <v>27</v>
       </c>
       <c r="J20" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>137</v>
@@ -2117,7 +2311,7 @@
         <v>27</v>
       </c>
       <c r="J21" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>143</v>
@@ -2161,7 +2355,7 @@
         <v>27</v>
       </c>
       <c r="J22" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>147</v>
@@ -2205,7 +2399,7 @@
         <v>27</v>
       </c>
       <c r="J23" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>151</v>
@@ -2249,7 +2443,7 @@
         <v>27</v>
       </c>
       <c r="J24" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>155</v>
@@ -2293,7 +2487,7 @@
         <v>27</v>
       </c>
       <c r="J25" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K25" s="1" t="s">
         <v>158</v>
@@ -2337,7 +2531,7 @@
         <v>27</v>
       </c>
       <c r="J26" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K26" s="1" t="s">
         <v>165</v>
@@ -2381,7 +2575,7 @@
         <v>27</v>
       </c>
       <c r="J27" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>168</v>
@@ -2425,7 +2619,7 @@
         <v>27</v>
       </c>
       <c r="J28" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>171</v>
@@ -2469,7 +2663,7 @@
         <v>27</v>
       </c>
       <c r="J29" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>175</v>
@@ -2513,7 +2707,7 @@
         <v>78</v>
       </c>
       <c r="J30" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>183</v>
@@ -2557,7 +2751,7 @@
         <v>27</v>
       </c>
       <c r="J31" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>190</v>
@@ -2601,7 +2795,7 @@
         <v>78</v>
       </c>
       <c r="J32" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>197</v>
@@ -2645,7 +2839,7 @@
         <v>27</v>
       </c>
       <c r="J33" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>203</v>
@@ -2689,7 +2883,7 @@
         <v>27</v>
       </c>
       <c r="J34" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>210</v>
@@ -2733,7 +2927,7 @@
         <v>92</v>
       </c>
       <c r="J35" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>216</v>
@@ -2777,7 +2971,7 @@
         <v>27</v>
       </c>
       <c r="J36" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>219</v>
@@ -2821,7 +3015,7 @@
         <v>92</v>
       </c>
       <c r="J37" t="s">
-        <v>229</v>
+        <v>291</v>
       </c>
       <c r="K37" s="1" t="s">
         <v>226</v>
@@ -2832,8 +3026,496 @@
       <c r="M37" t="s">
         <v>227</v>
       </c>
+      <c r="O37" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>229</v>
+      </c>
+      <c r="B38" t="s">
+        <v>230</v>
+      </c>
+      <c r="C38" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" t="s">
+        <v>231</v>
+      </c>
+      <c r="F38" t="s">
+        <v>232</v>
+      </c>
+      <c r="G38" t="s">
+        <v>25</v>
+      </c>
+      <c r="H38" t="s">
+        <v>102</v>
+      </c>
+      <c r="I38" t="s">
+        <v>27</v>
+      </c>
+      <c r="J38" t="s">
+        <v>291</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="L38" t="s">
+        <v>233</v>
+      </c>
+      <c r="M38" t="s">
+        <v>234</v>
+      </c>
+      <c r="O38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>244</v>
+      </c>
+      <c r="B39" t="s">
+        <v>236</v>
+      </c>
+      <c r="C39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" t="s">
+        <v>22</v>
+      </c>
+      <c r="E39" t="s">
+        <v>237</v>
+      </c>
+      <c r="F39" t="s">
+        <v>238</v>
+      </c>
+      <c r="G39" t="s">
+        <v>239</v>
+      </c>
+      <c r="H39" t="s">
+        <v>102</v>
+      </c>
+      <c r="I39" t="s">
+        <v>27</v>
+      </c>
+      <c r="J39" t="s">
+        <v>291</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="L39" t="s">
+        <v>240</v>
+      </c>
+      <c r="M39" t="s">
+        <v>241</v>
+      </c>
+      <c r="O39" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>243</v>
+      </c>
+      <c r="B40" t="s">
+        <v>245</v>
+      </c>
+      <c r="C40" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" t="s">
+        <v>246</v>
+      </c>
+      <c r="F40" t="s">
+        <v>247</v>
+      </c>
+      <c r="G40" t="s">
+        <v>248</v>
+      </c>
+      <c r="H40" t="s">
+        <v>102</v>
+      </c>
+      <c r="I40" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" t="s">
+        <v>291</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="L40" t="s">
+        <v>250</v>
+      </c>
+      <c r="M40" t="s">
+        <v>251</v>
+      </c>
+      <c r="O40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>252</v>
+      </c>
+      <c r="B41" t="s">
+        <v>253</v>
+      </c>
+      <c r="C41" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" t="s">
+        <v>22</v>
+      </c>
+      <c r="E41" t="s">
+        <v>254</v>
+      </c>
+      <c r="F41" t="s">
+        <v>255</v>
+      </c>
+      <c r="G41" t="s">
+        <v>256</v>
+      </c>
+      <c r="H41" t="s">
+        <v>102</v>
+      </c>
+      <c r="I41" t="s">
+        <v>27</v>
+      </c>
+      <c r="J41" t="s">
+        <v>291</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="L41" t="s">
+        <v>258</v>
+      </c>
+      <c r="M41" t="s">
+        <v>241</v>
+      </c>
+      <c r="O41" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>259</v>
+      </c>
+      <c r="B42" t="s">
+        <v>260</v>
+      </c>
+      <c r="C42" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" t="s">
+        <v>261</v>
+      </c>
+      <c r="F42" t="s">
+        <v>262</v>
+      </c>
+      <c r="G42" t="s">
+        <v>263</v>
+      </c>
+      <c r="H42" t="s">
+        <v>102</v>
+      </c>
+      <c r="I42" t="s">
+        <v>27</v>
+      </c>
+      <c r="J42" t="s">
+        <v>291</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="L42" t="s">
+        <v>258</v>
+      </c>
+      <c r="M42" t="s">
+        <v>241</v>
+      </c>
+      <c r="O42" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>265</v>
+      </c>
+      <c r="B43" t="s">
+        <v>266</v>
+      </c>
+      <c r="C43" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" t="s">
+        <v>267</v>
+      </c>
+      <c r="F43" t="s">
+        <v>232</v>
+      </c>
+      <c r="G43" t="s">
+        <v>268</v>
+      </c>
+      <c r="H43" t="s">
+        <v>102</v>
+      </c>
+      <c r="I43" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" t="s">
+        <v>291</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="L43" t="s">
+        <v>227</v>
+      </c>
+      <c r="M43" t="s">
+        <v>234</v>
+      </c>
+      <c r="O43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>270</v>
+      </c>
+      <c r="B44" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" t="s">
+        <v>22</v>
+      </c>
+      <c r="E44" t="s">
+        <v>272</v>
+      </c>
+      <c r="F44" t="s">
+        <v>255</v>
+      </c>
+      <c r="G44" t="s">
+        <v>273</v>
+      </c>
+      <c r="H44" t="s">
+        <v>102</v>
+      </c>
+      <c r="I44" t="s">
+        <v>27</v>
+      </c>
+      <c r="J44" t="s">
+        <v>291</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L44" t="s">
+        <v>227</v>
+      </c>
+      <c r="M44" t="s">
+        <v>234</v>
+      </c>
+      <c r="O44" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>275</v>
+      </c>
+      <c r="B45" t="s">
+        <v>276</v>
+      </c>
+      <c r="C45" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" t="s">
+        <v>277</v>
+      </c>
+      <c r="E45" t="s">
+        <v>278</v>
+      </c>
+      <c r="F45" t="s">
+        <v>279</v>
+      </c>
+      <c r="G45" t="s">
+        <v>280</v>
+      </c>
+      <c r="H45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I45" t="s">
+        <v>27</v>
+      </c>
+      <c r="J45" t="s">
+        <v>291</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="L45" t="s">
+        <v>227</v>
+      </c>
+      <c r="M45" t="s">
+        <v>234</v>
+      </c>
+      <c r="O45" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>282</v>
+      </c>
+      <c r="B46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C46" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" t="s">
+        <v>277</v>
+      </c>
+      <c r="E46" t="s">
+        <v>278</v>
+      </c>
+      <c r="F46" t="s">
+        <v>279</v>
+      </c>
+      <c r="G46" t="s">
+        <v>280</v>
+      </c>
+      <c r="H46" t="s">
+        <v>225</v>
+      </c>
+      <c r="I46" t="s">
+        <v>27</v>
+      </c>
+      <c r="J46" t="s">
+        <v>291</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="L46" t="s">
+        <v>227</v>
+      </c>
+      <c r="M46" t="s">
+        <v>234</v>
+      </c>
+      <c r="O46" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>284</v>
+      </c>
+      <c r="B47" t="s">
+        <v>285</v>
+      </c>
+      <c r="C47" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" t="s">
+        <v>286</v>
+      </c>
+      <c r="E47" t="s">
+        <v>278</v>
+      </c>
+      <c r="F47" t="s">
+        <v>279</v>
+      </c>
+      <c r="G47" t="s">
+        <v>280</v>
+      </c>
+      <c r="H47" t="s">
+        <v>225</v>
+      </c>
+      <c r="I47" t="s">
+        <v>27</v>
+      </c>
+      <c r="J47" t="s">
+        <v>291</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="L47" t="s">
+        <v>227</v>
+      </c>
+      <c r="M47" t="s">
+        <v>234</v>
+      </c>
+      <c r="O47" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>287</v>
+      </c>
+      <c r="B48" t="s">
+        <v>276</v>
+      </c>
+      <c r="C48" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" t="s">
+        <v>288</v>
+      </c>
+      <c r="F48" t="s">
+        <v>289</v>
+      </c>
+      <c r="G48" t="s">
+        <v>290</v>
+      </c>
+      <c r="H48" t="s">
+        <v>102</v>
+      </c>
+      <c r="I48" t="s">
+        <v>27</v>
+      </c>
+      <c r="J48" t="s">
+        <v>291</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="L48" t="s">
+        <v>227</v>
+      </c>
+      <c r="M48" t="s">
+        <v>234</v>
+      </c>
+      <c r="O48" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="K2" r:id="rId1" xr:uid="{7FC909CC-855C-47A2-BBD0-02C6480FC499}"/>
     <hyperlink ref="K3" r:id="rId2" xr:uid="{90EE97AC-5F97-4EC0-BC67-B270378001A0}"/>
@@ -2871,9 +3553,20 @@
     <hyperlink ref="K35" r:id="rId34" xr:uid="{1C3C2FF2-5376-42EF-93F4-40745ADD3F65}"/>
     <hyperlink ref="K36" r:id="rId35" xr:uid="{ABBA607B-E98F-4ACC-8057-5D87EC06529B}"/>
     <hyperlink ref="K37" r:id="rId36" xr:uid="{0CD417ED-9BF5-49B0-AC38-D13323646B78}"/>
+    <hyperlink ref="K38" r:id="rId37" xr:uid="{1330E8E9-4222-4D99-B471-A762D4C7BFAC}"/>
+    <hyperlink ref="K39" r:id="rId38" xr:uid="{50060393-6BFC-4AC4-AF68-1ACFE2D6968D}"/>
+    <hyperlink ref="K40" r:id="rId39" xr:uid="{635C6B86-5D7B-4A41-9D27-35645A2FCE58}"/>
+    <hyperlink ref="K41" r:id="rId40" xr:uid="{F22F0192-C6FD-4F79-A5BB-C783A98AA63F}"/>
+    <hyperlink ref="K42" r:id="rId41" xr:uid="{B53ED3B7-DF00-4A91-ACCE-D3E1DF8E0701}"/>
+    <hyperlink ref="K43" r:id="rId42" xr:uid="{8EFD53FB-6004-417A-BCAC-EDA986B42EBA}"/>
+    <hyperlink ref="K44" r:id="rId43" xr:uid="{C694EF44-24D5-4C81-B3F3-84EC2FA257A8}"/>
+    <hyperlink ref="K45" r:id="rId44" xr:uid="{F5F2046E-DAFA-4882-9C02-CD9B7B2205FB}"/>
+    <hyperlink ref="K46" r:id="rId45" xr:uid="{40DD3EE0-6088-4B53-8388-97F73D11D568}"/>
+    <hyperlink ref="K47" r:id="rId46" xr:uid="{40C4B132-A36D-4CCA-B235-B95BFDB53804}"/>
+    <hyperlink ref="K48" r:id="rId47" xr:uid="{10A9C74A-0A64-4B21-BC9B-D76B5DCE8C6F}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId48"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: admin dashboard updates, doctor modules, customer improvements
</commit_message>
<xml_diff>
--- a/docs/qa_guides/Frontend_Bugs_and_Refactoring_Template(AutoRecovered).xlsx
+++ b/docs/qa_guides/Frontend_Bugs_and_Refactoring_Template(AutoRecovered).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1.STUDY\FYP\Main\Philbox\docs\qa_guides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC70E29-6C17-4DDA-82FE-7D2D59B0265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212CB794-5C34-42FF-A33F-AD93DA3B9F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1390,7 +1390,9 @@
     <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="13" width="25" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="91.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="25" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>

</xml_diff>